<commit_message>
Add solutions to the alloy mixing problem
</commit_message>
<xml_diff>
--- a/excel/Alloys-Solution.xlsx
+++ b/excel/Alloys-Solution.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boyko\stats\opt2025\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Boyko Amarov\stats\opt2026\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E4BFF1F-4CBA-45CA-9E01-4AFF376A2B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D57EC11C-0577-4BD0-8393-4D14E19E38F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{9F0949AA-8545-4911-8F65-5FCD997E7D4F}"/>
+    <workbookView xWindow="18855" yWindow="7095" windowWidth="22725" windowHeight="11760" activeTab="2" xr2:uid="{9F0949AA-8545-4911-8F65-5FCD997E7D4F}"/>
   </bookViews>
   <sheets>
     <sheet name="Answer Report 1" sheetId="2" r:id="rId1"/>
@@ -123,9 +123,6 @@
     <t>Cost USD/kg</t>
   </si>
   <si>
-    <t>Usage</t>
-  </si>
-  <si>
     <t>Cost</t>
   </si>
   <si>
@@ -346,6 +343,9 @@
   </si>
   <si>
     <t>R.H. Side</t>
+  </si>
+  <si>
+    <t>Share</t>
   </si>
 </sst>
 </file>
@@ -377,12 +377,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -446,23 +452,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -798,383 +803,383 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45699E57-46E3-443D-B9CC-701A793F7FAF}">
   <dimension ref="A1:G37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.33203125" customWidth="1"/>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
     <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B11" t="s">
+    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="3" t="s">
+    </row>
+    <row r="16" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="2">
+        <v>6.1</v>
+      </c>
+      <c r="E16" s="2">
+        <v>4.9800000000000004</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="2" t="s">
+    <row r="20" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B21" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="5">
-        <v>6.1</v>
-      </c>
-      <c r="E16" s="5">
-        <v>4.9800000000000004</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="3" t="s">
+      <c r="C21" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="E21" s="4">
+        <v>1.6653345369377348E-16</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="4">
+        <v>0.2</v>
+      </c>
+      <c r="E22" s="4">
+        <v>0.59999999999999976</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B24" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" s="4">
+        <v>0</v>
+      </c>
+      <c r="E24" s="4">
+        <v>0.40000000000000008</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B25" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="4">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B26" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="4">
+        <v>0</v>
+      </c>
+      <c r="E26" s="4">
+        <v>0</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" s="4">
+        <v>0</v>
+      </c>
+      <c r="E27" s="4">
+        <v>0</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="4">
+        <v>0.7</v>
+      </c>
+      <c r="E28" s="4">
+        <v>0</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D29" s="2">
+        <v>0</v>
+      </c>
+      <c r="E29" s="2">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D21" s="6">
-        <v>0.1</v>
-      </c>
-      <c r="E21" s="6">
-        <v>1.6653345369377348E-16</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D22" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="E22" s="6">
-        <v>0.59999999999999976</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D23" s="6">
-        <v>0</v>
-      </c>
-      <c r="E23" s="6">
-        <v>0</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D24" s="6">
-        <v>0</v>
-      </c>
-      <c r="E24" s="6">
-        <v>0.40000000000000008</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" s="6">
-        <v>0</v>
-      </c>
-      <c r="E25" s="6">
-        <v>0</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D26" s="6">
-        <v>0</v>
-      </c>
-      <c r="E26" s="6">
-        <v>0</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="6">
-        <v>0</v>
-      </c>
-      <c r="E27" s="6">
-        <v>0</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D28" s="6">
-        <v>0.7</v>
-      </c>
-      <c r="E28" s="6">
-        <v>0</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C29" s="2" t="s">
+      <c r="D33" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="5">
-        <v>0</v>
-      </c>
-      <c r="E29" s="5">
-        <v>0</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D33" s="3" t="s">
+      <c r="C34" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D34" s="4">
+        <v>30</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G34" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B35" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D35" s="4">
+        <v>30</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G35" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D36" s="4">
         <v>40</v>
       </c>
-      <c r="E33" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B34" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D34" s="6">
-        <v>30</v>
-      </c>
-      <c r="E34" s="4" t="s">
+      <c r="E36" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F36" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F34" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G34" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B35" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="D35" s="6">
-        <v>30</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G35" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B36" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D36" s="6">
-        <v>40</v>
-      </c>
-      <c r="E36" s="4" t="s">
+      <c r="G36" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="F36" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G36" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2">
+        <v>1</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D37" s="5">
-        <v>1</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="F37" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G37" s="2">
         <v>0</v>
@@ -1188,85 +1193,85 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FB77635-A18F-489C-A8C8-6DAAA9AAD01F}">
   <dimension ref="A1:H25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.33203125" customWidth="1"/>
-    <col min="2" max="2" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.28515625" customWidth="1"/>
+    <col min="2" max="2" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E7" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="F7" s="7" t="s">
+      <c r="E8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G8" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="G8" s="8" t="s">
+      <c r="H8" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="H8" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="D9" s="4">
         <v>1.6653345369377348E-16</v>
@@ -1284,12 +1289,12 @@
         <v>0.28000000000000147</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>50</v>
       </c>
       <c r="D10" s="4">
         <v>0.59999999999999976</v>
@@ -1307,12 +1312,12 @@
         <v>1E+30</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>52</v>
       </c>
       <c r="D11" s="4">
         <v>0</v>
@@ -1330,12 +1335,12 @@
         <v>0.28000000000000141</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>54</v>
       </c>
       <c r="D12" s="4">
         <v>0.40000000000000008</v>
@@ -1353,12 +1358,12 @@
         <v>1E+30</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="D13" s="4">
         <v>0</v>
@@ -1376,12 +1381,12 @@
         <v>2.6199999999999983</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>58</v>
       </c>
       <c r="D14" s="4">
         <v>0</v>
@@ -1399,12 +1404,12 @@
         <v>2.4200000000000013</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>60</v>
       </c>
       <c r="D15" s="4">
         <v>0</v>
@@ -1422,12 +1427,12 @@
         <v>2.4199999999999977</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>61</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>62</v>
       </c>
       <c r="D16" s="4">
         <v>0</v>
@@ -1445,12 +1450,12 @@
         <v>1.1399999999999992</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="D17" s="2">
         <v>0</v>
@@ -1468,59 +1473,59 @@
         <v>2.6599999999999975</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G20" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E21" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F21" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="G21" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="H20" s="7" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="G21" s="8" t="s">
+      <c r="H21" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="H21" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="D22" s="4">
         <v>30</v>
@@ -1538,12 +1543,12 @@
         <v>1.3877787807814459E-15</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>70</v>
       </c>
       <c r="D23" s="4">
         <v>30</v>
@@ -1561,12 +1566,12 @@
         <v>1.3877787807814457E-15</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B24" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="D24" s="4">
         <v>40</v>
@@ -1584,12 +1589,12 @@
         <v>1.3877787807814455E-15</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="D25" s="2">
         <v>1</v>
@@ -1615,12 +1620,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B758131C-1B7F-408B-B54E-7DCB6FC3E4AA}">
   <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -1655,10 +1660,10 @@
         <v>11</v>
       </c>
       <c r="L1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1697,7 +1702,7 @@
         <v>30.000000000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1736,7 +1741,7 @@
         <v>29.999999999999993</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1775,7 +1780,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1818,35 +1823,35 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="9">
+        <v>90</v>
+      </c>
+      <c r="B6" s="7">
         <v>1.6653345369377299E-16</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="8">
         <v>0.59999999999999976</v>
       </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
+      <c r="D6" s="8">
+        <v>0</v>
+      </c>
+      <c r="E6" s="8">
         <v>0.40000000000000008</v>
       </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
+      <c r="F6" s="8">
+        <v>0</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0</v>
+      </c>
+      <c r="H6" s="8">
+        <v>0</v>
+      </c>
+      <c r="I6" s="8">
+        <v>0</v>
+      </c>
+      <c r="J6" s="8">
         <v>0</v>
       </c>
       <c r="K6">
@@ -1857,12 +1862,12 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K7" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="K7" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>